<commit_message>
Catálogo: 70 séries verificadas; 7 pendências do MVP restantes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -4424,7 +4424,7 @@
       </c>
       <c r="I7" s="16" t="n">
         <f aca="false">COUNTIF(Brasil!$L$6:$L$130,H7)</f>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="I8" s="16" t="n">
         <f aca="false">COUNTIF(Brasil!$L$6:$L$130,H8)</f>
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5820,7 +5820,7 @@
         <v>27</v>
       </c>
       <c r="L21" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M21" s="26" t="s">
         <v>160</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="L22" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M22" s="26" t="s">
         <v>167</v>
@@ -5902,7 +5902,7 @@
         <v>27</v>
       </c>
       <c r="L23" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M23" s="26" t="s">
         <v>171</v>
@@ -5984,7 +5984,7 @@
         <v>27</v>
       </c>
       <c r="L25" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M25" s="26" t="s">
         <v>180</v>
@@ -7990,7 +7990,7 @@
         <v>27</v>
       </c>
       <c r="L75" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M75" s="26" t="s">
         <v>390</v>
@@ -8031,7 +8031,7 @@
         <v>27</v>
       </c>
       <c r="L76" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M76" s="26" t="s">
         <v>394</v>
@@ -8470,7 +8470,7 @@
         <v>27</v>
       </c>
       <c r="L87" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M87" s="26" t="s">
         <v>439</v>

</xml_diff>

<commit_message>
Catálogo: séries dos EUA verificadas no FRED (2 códigos inválidos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3059" uniqueCount="1120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3060" uniqueCount="1121">
   <si>
     <t xml:space="preserve">Argus — Catálogo de Dados</t>
   </si>
@@ -2265,7 +2265,7 @@
     <t xml:space="preserve">BEA API</t>
   </si>
   <si>
-    <t xml:space="preserve">NIPA T10206 (a confirmar)</t>
+    <t xml:space="preserve">NIPA T10206</t>
   </si>
   <si>
     <t xml:space="preserve">US$ bi</t>
@@ -2400,7 +2400,7 @@
     <t xml:space="preserve">GACDFSA e equivalentes</t>
   </si>
   <si>
-    <t xml:space="preserve">Substituto gratuito do ISM</t>
+    <t xml:space="preserve">Código GACDFSA não existe no FRED (HTTP 400 na validação de 2026-10-04); localizar o código correto</t>
   </si>
   <si>
     <t xml:space="preserve">US-040</t>
@@ -2652,7 +2652,7 @@
     <t xml:space="preserve">NAR / FRED</t>
   </si>
   <si>
-    <t xml:space="preserve">FIXHAI (a confirmar)</t>
+    <t xml:space="preserve">FIXHAI</t>
   </si>
   <si>
     <t xml:space="preserve">US-061</t>
@@ -2694,7 +2694,7 @@
     <t xml:space="preserve">FRED (Z.1)</t>
   </si>
   <si>
-    <t xml:space="preserve">TNWBSHNO (a confirmar)</t>
+    <t xml:space="preserve">TNWBSHNO</t>
   </si>
   <si>
     <t xml:space="preserve">US-065</t>
@@ -2967,10 +2967,13 @@
     <t xml:space="preserve">FRED (EIA)</t>
   </si>
   <si>
-    <t xml:space="preserve">WCSSTUS1 (a confirmar)</t>
+    <t xml:space="preserve">WCSSTUS1</t>
   </si>
   <si>
     <t xml:space="preserve">Mil barris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código WCSSTUS1 não existe no FRED (HTTP 400 na validação de 2026-10-04); localizar o código correto</t>
   </si>
   <si>
     <t xml:space="preserve">US-088</t>
@@ -4424,7 +4427,7 @@
       </c>
       <c r="I7" s="16" t="n">
         <f aca="false">COUNTIF(Brasil!$L$6:$L$130,H7)</f>
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,7 +4459,7 @@
       </c>
       <c r="I8" s="16" t="n">
         <f aca="false">COUNTIF(Brasil!$L$6:$L$130,H8)</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4804,7 +4807,7 @@
       </c>
       <c r="I22" s="16" t="n">
         <f aca="false">COUNTIF(EUA!$L$6:$L$101,H22)</f>
-        <v>4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4836,7 +4839,7 @@
       </c>
       <c r="I23" s="16" t="n">
         <f aca="false">COUNTIF(EUA!$L$6:$L$101,H23)</f>
-        <v>56</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4868,7 +4871,7 @@
       </c>
       <c r="I24" s="16" t="n">
         <f aca="false">COUNTIF(EUA!$L$6:$L$101,H24)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8749,7 +8752,7 @@
         <v>27</v>
       </c>
       <c r="L94" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M94" s="26"/>
     </row>
@@ -10364,7 +10367,7 @@
         <v>29</v>
       </c>
       <c r="L6" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M6" s="26"/>
     </row>
@@ -10403,7 +10406,7 @@
         <v>29</v>
       </c>
       <c r="L7" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M7" s="26"/>
     </row>
@@ -10442,7 +10445,7 @@
         <v>29</v>
       </c>
       <c r="L8" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M8" s="26"/>
     </row>
@@ -10481,7 +10484,7 @@
         <v>29</v>
       </c>
       <c r="L9" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M9" s="26"/>
     </row>
@@ -10559,7 +10562,7 @@
         <v>29</v>
       </c>
       <c r="L11" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M11" s="26"/>
     </row>
@@ -10598,7 +10601,7 @@
         <v>29</v>
       </c>
       <c r="L12" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M12" s="26"/>
     </row>
@@ -10756,7 +10759,7 @@
         <v>29</v>
       </c>
       <c r="L16" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M16" s="26"/>
     </row>
@@ -10795,7 +10798,7 @@
         <v>29</v>
       </c>
       <c r="L17" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M17" s="26"/>
     </row>
@@ -10955,7 +10958,7 @@
         <v>29</v>
       </c>
       <c r="L21" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M21" s="26"/>
     </row>
@@ -11035,7 +11038,7 @@
         <v>29</v>
       </c>
       <c r="L23" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M23" s="26"/>
     </row>
@@ -11074,7 +11077,7 @@
         <v>29</v>
       </c>
       <c r="L24" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M24" s="26"/>
     </row>
@@ -11113,7 +11116,7 @@
         <v>29</v>
       </c>
       <c r="L25" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M25" s="26"/>
     </row>
@@ -11152,7 +11155,7 @@
         <v>29</v>
       </c>
       <c r="L26" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M26" s="26"/>
     </row>
@@ -11191,7 +11194,7 @@
         <v>29</v>
       </c>
       <c r="L27" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M27" s="26" t="s">
         <v>715</v>
@@ -11273,7 +11276,7 @@
         <v>29</v>
       </c>
       <c r="L29" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M29" s="26" t="s">
         <v>723</v>
@@ -11392,7 +11395,7 @@
         <v>29</v>
       </c>
       <c r="L32" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M32" s="26"/>
     </row>
@@ -11550,7 +11553,7 @@
         <v>29</v>
       </c>
       <c r="L36" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M36" s="26"/>
     </row>
@@ -11589,7 +11592,7 @@
         <v>29</v>
       </c>
       <c r="L37" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M37" s="26"/>
     </row>
@@ -11706,7 +11709,7 @@
         <v>29</v>
       </c>
       <c r="L40" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M40" s="26"/>
     </row>
@@ -11745,7 +11748,7 @@
         <v>29</v>
       </c>
       <c r="L41" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M41" s="26" t="s">
         <v>775</v>
@@ -11786,7 +11789,7 @@
         <v>29</v>
       </c>
       <c r="L42" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M42" s="26" t="s">
         <v>723</v>
@@ -11833,7 +11836,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="25" t="s">
         <v>786</v>
       </c>
@@ -11868,7 +11871,7 @@
         <v>29</v>
       </c>
       <c r="L44" s="26" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M44" s="26" t="s">
         <v>789</v>
@@ -11909,7 +11912,7 @@
         <v>29</v>
       </c>
       <c r="L45" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M45" s="26"/>
     </row>
@@ -11948,7 +11951,7 @@
         <v>29</v>
       </c>
       <c r="L46" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M46" s="26"/>
     </row>
@@ -12069,7 +12072,7 @@
         <v>29</v>
       </c>
       <c r="L49" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M49" s="26"/>
     </row>
@@ -12108,7 +12111,7 @@
         <v>29</v>
       </c>
       <c r="L50" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M50" s="26"/>
     </row>
@@ -12227,7 +12230,7 @@
         <v>29</v>
       </c>
       <c r="L53" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M53" s="26"/>
     </row>
@@ -12266,7 +12269,7 @@
         <v>29</v>
       </c>
       <c r="L54" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M54" s="26"/>
     </row>
@@ -12346,7 +12349,7 @@
         <v>29</v>
       </c>
       <c r="L56" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M56" s="26"/>
     </row>
@@ -12385,7 +12388,7 @@
         <v>29</v>
       </c>
       <c r="L57" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M57" s="26"/>
     </row>
@@ -12424,7 +12427,7 @@
         <v>29</v>
       </c>
       <c r="L58" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M58" s="26"/>
     </row>
@@ -12502,7 +12505,7 @@
         <v>29</v>
       </c>
       <c r="L60" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M60" s="26" t="s">
         <v>850</v>
@@ -12543,7 +12546,7 @@
         <v>29</v>
       </c>
       <c r="L61" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M61" s="26"/>
     </row>
@@ -12623,7 +12626,7 @@
         <v>29</v>
       </c>
       <c r="L63" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M63" s="26"/>
     </row>
@@ -12779,7 +12782,7 @@
         <v>29</v>
       </c>
       <c r="L67" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M67" s="26" t="s">
         <v>880</v>
@@ -12859,7 +12862,7 @@
         <v>29</v>
       </c>
       <c r="L69" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M69" s="26"/>
     </row>
@@ -12898,7 +12901,7 @@
         <v>29</v>
       </c>
       <c r="L70" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M70" s="26"/>
     </row>
@@ -12976,7 +12979,7 @@
         <v>29</v>
       </c>
       <c r="L72" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M72" s="26"/>
     </row>
@@ -13054,7 +13057,7 @@
         <v>29</v>
       </c>
       <c r="L74" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M74" s="26"/>
     </row>
@@ -13132,7 +13135,7 @@
         <v>29</v>
       </c>
       <c r="L76" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M76" s="26"/>
     </row>
@@ -13329,7 +13332,7 @@
         <v>29</v>
       </c>
       <c r="L81" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M81" s="26"/>
     </row>
@@ -13487,7 +13490,7 @@
         <v>29</v>
       </c>
       <c r="L85" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M85" s="26"/>
     </row>
@@ -13606,7 +13609,7 @@
         <v>29</v>
       </c>
       <c r="L88" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M88" s="26"/>
     </row>
@@ -13729,7 +13732,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="25" t="s">
         <v>974</v>
       </c>
@@ -13764,13 +13767,15 @@
         <v>29</v>
       </c>
       <c r="L92" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="M92" s="26"/>
+        <v>16</v>
+      </c>
+      <c r="M92" s="26" t="s">
+        <v>980</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="25" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="B93" s="26" t="s">
         <v>60</v>
@@ -13779,10 +13784,10 @@
         <v>448</v>
       </c>
       <c r="D93" s="27" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="E93" s="26" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="F93" s="26" t="s">
         <v>124</v>
@@ -13806,12 +13811,12 @@
         <v>20</v>
       </c>
       <c r="M93" s="26" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="25" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="B94" s="26" t="s">
         <v>60</v>
@@ -13820,13 +13825,13 @@
         <v>448</v>
       </c>
       <c r="D94" s="27" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="E94" s="26" t="s">
         <v>464</v>
       </c>
       <c r="F94" s="26" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="G94" s="26" t="s">
         <v>140</v>
@@ -13844,30 +13849,30 @@
         <v>29</v>
       </c>
       <c r="L94" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M94" s="26" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="25" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="B95" s="26" t="s">
         <v>61</v>
       </c>
       <c r="C95" s="26" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="D95" s="27" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="E95" s="26" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="F95" s="26" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="G95" s="26" t="s">
         <v>140</v>
@@ -13885,25 +13890,25 @@
         <v>29</v>
       </c>
       <c r="L95" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M95" s="26"/>
     </row>
     <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="25" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="B96" s="26" t="s">
         <v>61</v>
       </c>
       <c r="C96" s="26" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="D96" s="27" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="E96" s="26" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="F96" s="26" t="s">
         <v>124</v>
@@ -13930,7 +13935,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="25" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="B97" s="26" t="s">
         <v>61</v>
@@ -13939,13 +13944,13 @@
         <v>358</v>
       </c>
       <c r="D97" s="27" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="E97" s="26" t="s">
         <v>464</v>
       </c>
       <c r="F97" s="26" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="G97" s="26" t="s">
         <v>140</v>
@@ -13963,15 +13968,15 @@
         <v>29</v>
       </c>
       <c r="L97" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M97" s="26" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="25" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="B98" s="26" t="s">
         <v>61</v>
@@ -13980,13 +13985,13 @@
         <v>928</v>
       </c>
       <c r="D98" s="27" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="E98" s="26" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="F98" s="26" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="G98" s="26" t="s">
         <v>100</v>
@@ -14010,7 +14015,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="25" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="B99" s="26" t="s">
         <v>61</v>
@@ -14019,13 +14024,13 @@
         <v>358</v>
       </c>
       <c r="D99" s="27" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="E99" s="26" t="s">
         <v>200</v>
       </c>
       <c r="F99" s="26" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="G99" s="26" t="s">
         <v>140</v>
@@ -14049,22 +14054,22 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="25" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="B100" s="26" t="s">
         <v>61</v>
       </c>
       <c r="C100" s="26" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="D100" s="27" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="E100" s="26" t="s">
         <v>464</v>
       </c>
       <c r="F100" s="26" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="G100" s="26" t="s">
         <v>100</v>
@@ -14082,13 +14087,13 @@
         <v>29</v>
       </c>
       <c r="L100" s="26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M100" s="26"/>
     </row>
     <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="25" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="B101" s="26" t="s">
         <v>61</v>
@@ -14097,13 +14102,13 @@
         <v>531</v>
       </c>
       <c r="D101" s="27" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="E101" s="26" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="F101" s="26" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="G101" s="26" t="s">
         <v>140</v>
@@ -14124,7 +14129,7 @@
         <v>14</v>
       </c>
       <c r="M101" s="26" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
     </row>
   </sheetData>
@@ -14196,12 +14201,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14217,10 +14222,10 @@
         <v>65</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="D5" s="24" t="s">
         <v>67</v>
@@ -14234,56 +14239,56 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>27</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>29</v>
@@ -14292,33 +14297,33 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>27</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="D10" s="26" t="s">
         <v>22</v>
@@ -14327,61 +14332,61 @@
         <v>27</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>27</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>27</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>31</v>
@@ -14390,36 +14395,36 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="E14" s="26" t="s">
         <v>31</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="E15" s="26" t="s">
         <v>27</v>
@@ -14428,16 +14433,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="E16" s="26" t="s">
         <v>31</v>
@@ -14446,16 +14451,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="E17" s="26" t="s">
         <v>33</v>
@@ -14499,12 +14504,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14520,19 +14525,19 @@
         <v>67</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14540,59 +14545,59 @@
         <v>98</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>1082</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F7" s="26" t="s">
         <v>1079</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>1080</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>1075</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>1081</v>
-      </c>
-      <c r="E7" s="28" t="s">
-        <v>1077</v>
-      </c>
-      <c r="F7" s="26" t="s">
-        <v>1078</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14600,39 +14605,39 @@
         <v>76</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14640,19 +14645,19 @@
         <v>425</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14660,19 +14665,19 @@
         <v>291</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="E12" s="28" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14680,39 +14685,39 @@
         <v>548</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="E13" s="28" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F13" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D14" s="26" t="s">
         <v>124</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14723,156 +14728,156 @@
         <v>573</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="B17" s="26" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>1107</v>
+      </c>
+      <c r="E17" s="29" t="s">
         <v>1091</v>
       </c>
-      <c r="C17" s="26" t="s">
-        <v>1105</v>
-      </c>
-      <c r="D17" s="26" t="s">
-        <v>1106</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>1090</v>
-      </c>
       <c r="F17" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="B18" s="26" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E18" s="29" t="s">
         <v>1091</v>
       </c>
-      <c r="C18" s="26" t="s">
-        <v>1105</v>
-      </c>
-      <c r="D18" s="26" t="s">
-        <v>1108</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>1090</v>
-      </c>
       <c r="F18" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="B19" s="26" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>1112</v>
+      </c>
+      <c r="E19" s="29" t="s">
         <v>1091</v>
       </c>
-      <c r="C19" s="26" t="s">
-        <v>1110</v>
-      </c>
-      <c r="D19" s="26" t="s">
-        <v>1111</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>1090</v>
-      </c>
       <c r="F19" s="26" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="B22" s="26" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C22" s="26" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>1119</v>
+      </c>
+      <c r="E22" s="29" t="s">
         <v>1091</v>
       </c>
-      <c r="C22" s="26" t="s">
-        <v>1110</v>
-      </c>
-      <c r="D22" s="26" t="s">
-        <v>1118</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>1090</v>
-      </c>
       <c r="F22" s="26" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 1, passo 6a: adapter do Focus e sub-séries
O contrato de adapter aceita uma sub-série opcional (ex.: ano de
referência do Focus, reunião do Copom), gravada como '<id>@<sub>'.
Adapter Focus: mediana, base de cálculo 0, paginação OData, 12 meses
suavizada. Catálogo: nomes oficiais dos indicadores fiscais e IPCA 12m.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -972,10 +972,10 @@
     <t xml:space="preserve">Focus — IPCA 12 meses à frente</t>
   </si>
   <si>
-    <t xml:space="preserve">ExpectativasMercadoInflacao12Meses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usado no juro real ex-ante</t>
+    <t xml:space="preserve">ExpectativasMercadoInflacao12Meses · Indicador='IPCA'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Série suavizada; usada no juro real ex-ante</t>
   </si>
   <si>
     <t xml:space="preserve">BR-048</t>
@@ -1359,7 +1359,7 @@
     <t xml:space="preserve">Focus — primário e dívida líquida</t>
   </si>
   <si>
-    <t xml:space="preserve">ExpectativasMercadoAnuais</t>
+    <t xml:space="preserve">ExpectativasMercadoAnuais · Indicador='Resultado primário' ; Indicador='Dívida líquida do setor público'</t>
   </si>
   <si>
     <t xml:space="preserve">BR-078</t>
@@ -8590,7 +8590,7 @@
       </c>
       <c r="M87" s="26"/>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="25" t="s">
         <v>439</v>
       </c>

</xml_diff>

<commit_message>
Catálogo: recortes do ComexStat (fluxos e destinos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -7424,7 +7424,7 @@
       </c>
       <c r="F90" s="26" t="inlineStr">
         <is>
-          <t>POST api-comexstat.mdic.gov.br/general</t>
+          <t>fluxo=export ; fluxo=import</t>
         </is>
       </c>
       <c r="G90" s="26" t="inlineStr">
@@ -7434,7 +7434,7 @@
       </c>
       <c r="H90" s="26" t="inlineStr">
         <is>
-          <t>US$ mi</t>
+          <t>US$ FOB</t>
         </is>
       </c>
       <c r="I90" s="26" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="D91" s="27" t="inlineStr">
         <is>
-          <t>Exportações por produto e destino (China, EUA, UE)</t>
+          <t>Exportações por destino (China, EUA, UE)</t>
         </is>
       </c>
       <c r="E91" s="26" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="F91" s="26" t="inlineStr">
         <is>
-          <t>POST api-comexstat.mdic.gov.br/general (por NCM/país)</t>
+          <t>fluxo=export/pais=160 ; fluxo=export/pais=249 ; fluxo=export/bloco=22</t>
         </is>
       </c>
       <c r="G91" s="26" t="inlineStr">
@@ -7501,7 +7501,7 @@
       </c>
       <c r="H91" s="26" t="inlineStr">
         <is>
-          <t>US$ mi</t>
+          <t>US$ FOB</t>
         </is>
       </c>
       <c r="I91" s="26" t="inlineStr">
@@ -7526,7 +7526,7 @@
       </c>
       <c r="M91" s="26" t="inlineStr">
         <is>
-          <t>Exposição a China e tarifas</t>
+          <t>Exposição a China e tarifas; Abertura por produto (SH4/NCM) fica para a v2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Decisão 0010 e catálogo: RTN pela API do Tesouro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -7096,12 +7096,12 @@
       </c>
       <c r="E85" s="26" t="inlineStr">
         <is>
-          <t>Tesouro Transparente</t>
+          <t>Tesouro Nacional (API RTN)</t>
         </is>
       </c>
       <c r="F85" s="26" t="inlineStr">
         <is>
-          <t>CKAN resultado-do-tesouro-nacional (XLSX série histórica)</t>
+          <t>rtn=10.01.1 ; rtn=10.02.1 ; rtn=10.01.2 ; rtn=10.03.1 ; rtn=10.04.1 ; rtn=10.08.1 ; rtn=10.09.1</t>
         </is>
       </c>
       <c r="G85" s="26" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="M85" s="26" t="inlineStr">
         <is>
-          <t>Planilha atualizada em 2026-08-27; layout mutável, teste de contrato obrigatório</t>
+          <t>API Séries Temporais do RTN (decisão 0010): receita total, transferências, receita líquida, despesa total, primário, juros e nominal; R$ milhões correntes</t>
         </is>
       </c>
     </row>
@@ -17522,7 +17522,7 @@
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>CKAN / CSV / xlsx</t>
+          <t>API Séries Temporais (RTN, JSON) · CKAN / xlsx</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
@@ -17532,12 +17532,12 @@
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>RTN e RMD em planilhas com layout mutável</t>
-        </is>
-      </c>
-      <c r="E12" s="28" t="inlineStr">
-        <is>
-          <t>Médio</t>
+          <t>RTN por API JSON paginada (decisão 0010); RMD ainda em planilha</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="F12" s="26" t="inlineStr">

</xml_diff>

<commit_message>
Catálogo: Ibovespa com código estruturado e início em 1998
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -9169,7 +9169,7 @@
       </c>
       <c r="F117" s="26" t="inlineStr">
         <is>
-          <t>B3 IndexCall/GetPortfolioDay IBOV · Yahoo ^BVSP</t>
+          <t>indice=IBOV · yahoo=^BVSP</t>
         </is>
       </c>
       <c r="G117" s="26" t="inlineStr">
@@ -9204,7 +9204,7 @@
       </c>
       <c r="M117" s="26" t="inlineStr">
         <is>
-          <t>FMP grátis não inclui Ibovespa (HTTP 402); SGS 7 descontinuada em 2019</t>
+          <t>Fechamento diário desde 1998 (antes, reescalonamentos ÷10 sem ajuste na fonte: v2). Yahoo cobre a janela recente se a B3 falhar; FMP grátis não inclui Ibovespa (HTTP 402)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catálogo: comunicados e atas do Copom com código estruturado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -6065,7 +6065,7 @@
       </c>
       <c r="F69" s="26" t="inlineStr">
         <is>
-          <t>api/servico/sitebcb/copom/comunicados · /atas</t>
+          <t>comunicados ; atas</t>
         </is>
       </c>
       <c r="G69" s="26" t="inlineStr">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="M69" s="26" t="inlineStr">
         <is>
-          <t>API do site, não documentada; respondeu com a 281ª reunião (set/2026). Teste de contrato obrigatório</t>
+          <t>API do site do BCB, não documentada (copom/comunicados, copom/atas e *_detalhes); texto convertido para texto puro na tabela events; comunicados desde a 46ª reunião (2000)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catálogo: Focus Selic anual (insumo do neutro) e saldo do CAGED derivado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Fontes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$138</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EUA'!$A$5:$M$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Central'!$A$5:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fontes'!$A$5:$F$25</definedName>
@@ -993,19 +993,19 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A7,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A7,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A7,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A7,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F7" s="6">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="I7" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$136,H7)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$138,H7)</f>
         <v/>
       </c>
     </row>
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A8,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A8,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A8,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A8,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F8" s="6">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="I8" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$136,H8)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$138,H8)</f>
         <v/>
       </c>
     </row>
@@ -1065,19 +1065,19 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A9,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A9,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A9,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A9,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F9" s="6">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="I9" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$136,H9)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$138,H9)</f>
         <v/>
       </c>
     </row>
@@ -1101,19 +1101,19 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A10,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A10,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A10,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A10,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F10" s="6">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="I10" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$136,H10)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$138,H10)</f>
         <v/>
       </c>
     </row>
@@ -1137,19 +1137,19 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A11,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A11,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A11,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A11,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F11" s="6">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="I11" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$136,H11)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$138,H11)</f>
         <v/>
       </c>
     </row>
@@ -1173,19 +1173,19 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A12,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A12,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A12,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A12,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F12" s="6">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="I12" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$136,H12)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$138,H12)</f>
         <v/>
       </c>
     </row>
@@ -1209,19 +1209,19 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A13,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A13,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A13,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A13,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F13" s="6">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="I13" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$136,H13)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$138,H13)</f>
         <v/>
       </c>
     </row>
@@ -1245,19 +1245,19 @@
         </is>
       </c>
       <c r="B14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A14,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A14,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A14,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A14,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F14" s="6">
@@ -1272,19 +1272,19 @@
         </is>
       </c>
       <c r="B15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A15,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A15,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A15,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A15,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F15" s="6">
@@ -1299,19 +1299,19 @@
         </is>
       </c>
       <c r="B16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A16,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A16,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A16,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A16,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F16" s="6">
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A17,Brasil!$K$6:$K$136,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"MVP")</f>
         <v/>
       </c>
       <c r="C17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A17,Brasil!$K$6:$K$136,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"EUA")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A17,Brasil!$K$6:$K$136,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"v2")</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$136,$A17,Brasil!$K$6:$K$136,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"v3")</f>
         <v/>
       </c>
       <c r="F17" s="6">
@@ -1766,7 +1766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M136"/>
+  <dimension ref="A1:M138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10441,9 +10441,143 @@
       </c>
       <c r="M136" s="26" t="inlineStr"/>
     </row>
+    <row r="137">
+      <c r="A137" s="25" t="inlineStr">
+        <is>
+          <t>BR-132</t>
+        </is>
+      </c>
+      <c r="B137" s="26" t="inlineStr">
+        <is>
+          <t>Política Monetária</t>
+        </is>
+      </c>
+      <c r="C137" s="26" t="inlineStr">
+        <is>
+          <t>Expectativas</t>
+        </is>
+      </c>
+      <c r="D137" s="27" t="inlineStr">
+        <is>
+          <t>Focus — Selic fim de ano (ano corrente a +3)</t>
+        </is>
+      </c>
+      <c r="E137" s="26" t="inlineStr">
+        <is>
+          <t>BCB Olinda (Focus)</t>
+        </is>
+      </c>
+      <c r="F137" s="26" t="inlineStr">
+        <is>
+          <t>ExpectativasMercadoAnuais · Indicador='Selic'</t>
+        </is>
+      </c>
+      <c r="G137" s="26" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="H137" s="26" t="inlineStr">
+        <is>
+          <t>% a.a.</t>
+        </is>
+      </c>
+      <c r="I137" s="26" t="inlineStr">
+        <is>
+          <t>Taxa</t>
+        </is>
+      </c>
+      <c r="J137" s="26" t="inlineStr">
+        <is>
+          <t>Nível, Δ p.p. (MoM, YoY, 3/6/12m)</t>
+        </is>
+      </c>
+      <c r="K137" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L137" s="26" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="M137" s="26" t="inlineStr">
+        <is>
+          <t>Insumo do juro neutro implícito (BR-117); sub-série por ano de referência</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="25" t="inlineStr">
+        <is>
+          <t>BR-133</t>
+        </is>
+      </c>
+      <c r="B138" s="26" t="inlineStr">
+        <is>
+          <t>Mercado de Trabalho</t>
+        </is>
+      </c>
+      <c r="C138" s="26" t="inlineStr">
+        <is>
+          <t>Formal</t>
+        </is>
+      </c>
+      <c r="D138" s="27" t="inlineStr">
+        <is>
+          <t>Saldo mensal do Novo CAGED (variação do estoque)</t>
+        </is>
+      </c>
+      <c r="E138" s="26" t="inlineStr">
+        <is>
+          <t>Argus</t>
+        </is>
+      </c>
+      <c r="F138" s="26" t="inlineStr">
+        <is>
+          <t>Δ(28763)</t>
+        </is>
+      </c>
+      <c r="G138" s="26" t="inlineStr">
+        <is>
+          <t>Mensal</t>
+        </is>
+      </c>
+      <c r="H138" s="26" t="inlineStr">
+        <is>
+          <t>Postos</t>
+        </is>
+      </c>
+      <c r="I138" s="26" t="inlineStr">
+        <is>
+          <t>Derivado</t>
+        </is>
+      </c>
+      <c r="J138" s="26" t="inlineStr">
+        <is>
+          <t>Nível, soma 3/12m, MoM % (SA), YoY %, real/nominal, % PIB</t>
+        </is>
+      </c>
+      <c r="K138" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L138" s="26" t="inlineStr">
+        <is>
+          <t>Derivado</t>
+        </is>
+      </c>
+      <c r="M138" s="26" t="inlineStr">
+        <is>
+          <t>Variação mensal do estoque BR-022; só entre meses consecutivos</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:M136"/>
-  <conditionalFormatting sqref="L6:L336">
+  <autoFilter ref="A5:M138"/>
+  <conditionalFormatting sqref="L6:L338">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L6="Verificado"</formula>
     </cfRule>
@@ -10466,16 +10600,16 @@
       <formula>$L6="Curado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K336">
+  <conditionalFormatting sqref="K6:K338">
     <cfRule type="expression" priority="8" dxfId="7">
       <formula>$K6="MVP"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K6:K336" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K338" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MVP,EUA,v2,v3"</formula1>
     </dataValidation>
-    <dataValidation sqref="L6:L336" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L6:L338" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Verificado,Confirmar,A mapear,Sem API,Pago,Derivado,Curado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Catálogo: Focus Selic anual verificado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -10499,12 +10499,12 @@
       </c>
       <c r="L137" s="26" t="inlineStr">
         <is>
-          <t>Confirmar</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="M137" s="26" t="inlineStr">
         <is>
-          <t>Insumo do juro neutro implícito (BR-117); sub-série por ano de referência</t>
+          <t>Insumo do juro neutro implícito (BR-117); sub-série por ano de referência; validador 2026-10-04: última pesquisa 2026-09-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catálogo: serviços e industriais subjacentes passam a ser séries oficiais do SGS (NT 57); EX2 = 27838
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -3961,7 +3961,7 @@
       </c>
       <c r="F37" s="26" t="inlineStr">
         <is>
-          <t>16121</t>
+          <t>27838</t>
         </is>
       </c>
       <c r="G37" s="26" t="inlineStr">
@@ -3991,12 +3991,12 @@
       </c>
       <c r="L37" s="26" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Confirmar</t>
         </is>
       </c>
       <c r="M37" s="26" t="inlineStr">
         <is>
-          <t>Há dois códigos com título EX2: 16121 ("ex2") e 27838 ("EX2"); confirmar qual é a série vigente antes da Fase 3</t>
+          <t>NT 57 (dez/2025, Tabela 11): EX1 = 16121 e EX2 = 27838; o título SGS de 16121 ('ex2') é enganoso</t>
         </is>
       </c>
     </row>
@@ -4349,17 +4349,17 @@
       </c>
       <c r="D43" s="27" t="inlineStr">
         <is>
-          <t>Bens industriais subjacentes</t>
+          <t>Bens industriais subjacentes (EX3 Industriais)</t>
         </is>
       </c>
       <c r="E43" s="26" t="inlineStr">
         <is>
-          <t>Argus</t>
+          <t>BCB SGS</t>
         </is>
       </c>
       <c r="F43" s="26" t="inlineStr">
         <is>
-          <t>f(t7060): metodologia BCB (industriais ex-voláteis)</t>
+          <t>29684</t>
         </is>
       </c>
       <c r="G43" s="26" t="inlineStr">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="I43" s="26" t="inlineStr">
         <is>
-          <t>Derivado</t>
+          <t>Var % mensal</t>
         </is>
       </c>
       <c r="J43" s="26" t="inlineStr">
@@ -4389,12 +4389,12 @@
       </c>
       <c r="L43" s="26" t="inlineStr">
         <is>
-          <t>Derivado</t>
+          <t>Confirmar</t>
         </is>
       </c>
       <c r="M43" s="26" t="inlineStr">
         <is>
-          <t>Par de serviços subjacentes; conferir contra boxes do RPM</t>
+          <t>Série oficial do BCB desde a NT 57 (dez/2025, Tabela 11): antes era cálculo próprio</t>
         </is>
       </c>
     </row>
@@ -4995,17 +4995,17 @@
       </c>
       <c r="D53" s="27" t="inlineStr">
         <is>
-          <t>Serviços subjacentes / supercore BR</t>
+          <t>Serviços subjacentes (EX3 Serviços)</t>
         </is>
       </c>
       <c r="E53" s="26" t="inlineStr">
         <is>
-          <t>Argus</t>
+          <t>BCB SGS</t>
         </is>
       </c>
       <c r="F53" s="26" t="inlineStr">
         <is>
-          <t>f(t7060)</t>
+          <t>29683</t>
         </is>
       </c>
       <c r="G53" s="26" t="inlineStr">
@@ -5020,12 +5020,12 @@
       </c>
       <c r="I53" s="26" t="inlineStr">
         <is>
-          <t>Derivado</t>
+          <t>Var % mensal</t>
         </is>
       </c>
       <c r="J53" s="26" t="inlineStr">
         <is>
-          <t>Conforme definição da fórmula</t>
+          <t>Mensal, acum. 3/6/9/12m (encadeado), 3m/6m anualizado, YoY via 12m</t>
         </is>
       </c>
       <c r="K53" s="26" t="inlineStr">
@@ -5035,12 +5035,12 @@
       </c>
       <c r="L53" s="26" t="inlineStr">
         <is>
-          <t>Derivado</t>
+          <t>Confirmar</t>
         </is>
       </c>
       <c r="M53" s="26" t="inlineStr">
         <is>
-          <t>Recalcular com a metodologia do BCB e validar contra o RPM</t>
+          <t>Série oficial do BCB desde a NT 57 (dez/2025, Tabela 11): antes era cálculo próprio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catálogo: EX2, serviços e industriais subjacentes verificados; P50 com método conferido
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -3991,12 +3991,12 @@
       </c>
       <c r="L37" s="26" t="inlineStr">
         <is>
-          <t>Confirmar</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="M37" s="26" t="inlineStr">
         <is>
-          <t>NT 57 (dez/2025, Tabela 11): EX1 = 16121 e EX2 = 27838; o título SGS de 16121 ('ex2') é enganoso</t>
+          <t>NT 57 (dez/2025, Tabela 11): EX1 = 16121 e EX2 = 27838; o título SGS de 16121 ('ex2') é enganoso; validador 2026-10-04: título oficial confere</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="M42" s="26" t="inlineStr">
         <is>
-          <t>Complementa o P55 oficial; documentar metodologia em docs/metodologia</t>
+          <t>Método do P55 do BCB (NT 57) em 50%; o mesmo cálculo em 55% reproduz o SGS 28750 em 80 de 80 meses (2020-2026). Desde 2020 (tabela 7060)</t>
         </is>
       </c>
     </row>
@@ -4389,12 +4389,12 @@
       </c>
       <c r="L43" s="26" t="inlineStr">
         <is>
-          <t>Confirmar</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="M43" s="26" t="inlineStr">
         <is>
-          <t>Série oficial do BCB desde a NT 57 (dez/2025, Tabela 11): antes era cálculo próprio</t>
+          <t>Série oficial do BCB desde a NT 57 (dez/2025, Tabela 11): antes era cálculo próprio; validador 2026-10-04: título oficial confere</t>
         </is>
       </c>
     </row>
@@ -5035,12 +5035,12 @@
       </c>
       <c r="L53" s="26" t="inlineStr">
         <is>
-          <t>Confirmar</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="M53" s="26" t="inlineStr">
         <is>
-          <t>Série oficial do BCB desde a NT 57 (dez/2025, Tabela 11): antes era cálculo próprio</t>
+          <t>Série oficial do BCB desde a NT 57 (dez/2025, Tabela 11): antes era cálculo próprio; validador 2026-10-04: título oficial confere</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 2, passo 1b: recortes oficiais do IBGE para conferir as transformações; decisão 0012 e spec aprovada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -2306,7 +2306,7 @@
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>t8888/v12606,12607/c544=129314,129315,129316</t>
+          <t>t8888/v12606,12607/c544=129314,129315,129316 ; t8888/v11602,11604/c544=129314</t>
         </is>
       </c>
       <c r="G12" s="26" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="M12" s="26" t="inlineStr">
         <is>
-          <t>Tabela nova (base 2022); conferir na Fase 0</t>
+          <t>Tabela nova (base 2022); conferir na Fase 0; v11602 (YoY) e v11604 (12 meses) são as taxas oficiais, usadas para conferir o cálculo do site</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>t8880/v7169,7170/c11046=56733,56734 ; t8881/v7169,7170/c11046=56735,56736</t>
+          <t>t8880/v7169,7170/c11046=56733,56734 ; t8881/v7169,7170/c11046=56735,56736 ; t8880/v11708/c11046=56734</t>
         </is>
       </c>
       <c r="G13" s="26" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="M13" s="26" t="inlineStr">
         <is>
-          <t>Volume e receita nominal</t>
+          <t>Volume e receita nominal; t8880 v11708 (MoM SA oficial) confere o cálculo do site</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catálogo: meta para a inflação (BR-134, SGS 13521)
Título oficial conferido no SGS; insumo da regra de Taylor e do desvio da meta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Fontes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EUA'!$A$5:$M$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Central'!$A$5:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fontes'!$A$5:$F$25</definedName>
@@ -993,19 +993,19 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A7,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F7" s="6">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="I7" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$138,H7)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$139,H7)</f>
         <v/>
       </c>
     </row>
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A8,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F8" s="6">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="I8" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$138,H8)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$139,H8)</f>
         <v/>
       </c>
     </row>
@@ -1065,19 +1065,19 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A9,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F9" s="6">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="I9" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$138,H9)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$139,H9)</f>
         <v/>
       </c>
     </row>
@@ -1101,19 +1101,19 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A10,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F10" s="6">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="I10" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$138,H10)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$139,H10)</f>
         <v/>
       </c>
     </row>
@@ -1137,19 +1137,19 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A11,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F11" s="6">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="I11" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$138,H11)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$139,H11)</f>
         <v/>
       </c>
     </row>
@@ -1173,19 +1173,19 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A12,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F12" s="6">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="I12" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$138,H12)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$139,H12)</f>
         <v/>
       </c>
     </row>
@@ -1209,19 +1209,19 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A13,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F13" s="6">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="I13" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$138,H13)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$139,H13)</f>
         <v/>
       </c>
     </row>
@@ -1245,19 +1245,19 @@
         </is>
       </c>
       <c r="B14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A14,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F14" s="6">
@@ -1272,19 +1272,19 @@
         </is>
       </c>
       <c r="B15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A15,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F15" s="6">
@@ -1299,19 +1299,19 @@
         </is>
       </c>
       <c r="B16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A16,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F16" s="6">
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"MVP")</f>
         <v/>
       </c>
       <c r="C17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"EUA")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"v2")</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$138,$A17,Brasil!$K$6:$K$138,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"v3")</f>
         <v/>
       </c>
       <c r="F17" s="6">
@@ -1766,7 +1766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M138"/>
+  <dimension ref="A1:M139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10575,9 +10575,76 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="25" t="inlineStr">
+        <is>
+          <t>BR-134</t>
+        </is>
+      </c>
+      <c r="B139" s="26" t="inlineStr">
+        <is>
+          <t>Inflação</t>
+        </is>
+      </c>
+      <c r="C139" s="26" t="inlineStr">
+        <is>
+          <t>Cheio</t>
+        </is>
+      </c>
+      <c r="D139" s="27" t="inlineStr">
+        <is>
+          <t>Meta para a inflação (CMN)</t>
+        </is>
+      </c>
+      <c r="E139" s="26" t="inlineStr">
+        <is>
+          <t>BCB SGS</t>
+        </is>
+      </c>
+      <c r="F139" s="26" t="inlineStr">
+        <is>
+          <t>13521</t>
+        </is>
+      </c>
+      <c r="G139" s="26" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="H139" s="26" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I139" s="26" t="inlineStr">
+        <is>
+          <t>Taxa</t>
+        </is>
+      </c>
+      <c r="J139" s="26" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="K139" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L139" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M139" s="26" t="inlineStr">
+        <is>
+          <t>Título oficial 'Meta para a inflação' conferido em 2026-10-15; valor central do ano (o intervalo de tolerância não está no SGS). Insumo da regra de Taylor e do desvio da meta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:M138"/>
-  <conditionalFormatting sqref="L6:L338">
+  <autoFilter ref="A5:M139"/>
+  <conditionalFormatting sqref="L6:L339">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L6="Verificado"</formula>
     </cfRule>
@@ -10600,16 +10667,16 @@
       <formula>$L6="Curado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K338">
+  <conditionalFormatting sqref="K6:K339">
     <cfRule type="expression" priority="8" dxfId="7">
       <formula>$K6="MVP"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K6:K338" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K339" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MVP,EUA,v2,v3"</formula1>
     </dataValidation>
-    <dataValidation sqref="L6:L338" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L6:L339" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Verificado,Confirmar,A mapear,Sem API,Pago,Derivado,Curado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Catálogo: classificações do IPCA do BCB (comercializáveis, não comercializáveis, duráveis, semiduráveis, não duráveis)
Títulos oficiais conferidos no SGS; base da seção Áreas de influência do IPCA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014U6sAweK8dE2VxgRNrvDsS
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Fontes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$144</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EUA'!$A$5:$M$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Central'!$A$5:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fontes'!$A$5:$F$25</definedName>
@@ -993,19 +993,19 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A7,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F7" s="6">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="I7" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$139,H7)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$144,H7)</f>
         <v/>
       </c>
     </row>
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A8,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F8" s="6">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="I8" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$139,H8)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$144,H8)</f>
         <v/>
       </c>
     </row>
@@ -1065,19 +1065,19 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A9,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F9" s="6">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="I9" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$139,H9)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$144,H9)</f>
         <v/>
       </c>
     </row>
@@ -1101,19 +1101,19 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A10,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F10" s="6">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="I10" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$139,H10)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$144,H10)</f>
         <v/>
       </c>
     </row>
@@ -1137,19 +1137,19 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A11,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F11" s="6">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="I11" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$139,H11)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$144,H11)</f>
         <v/>
       </c>
     </row>
@@ -1173,19 +1173,19 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A12,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F12" s="6">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="I12" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$139,H12)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$144,H12)</f>
         <v/>
       </c>
     </row>
@@ -1209,19 +1209,19 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A13,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F13" s="6">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="I13" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$139,H13)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$144,H13)</f>
         <v/>
       </c>
     </row>
@@ -1245,19 +1245,19 @@
         </is>
       </c>
       <c r="B14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A14,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F14" s="6">
@@ -1272,19 +1272,19 @@
         </is>
       </c>
       <c r="B15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A15,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F15" s="6">
@@ -1299,19 +1299,19 @@
         </is>
       </c>
       <c r="B16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A16,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F16" s="6">
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"MVP")</f>
         <v/>
       </c>
       <c r="C17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"EUA")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"v2")</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$139,$A17,Brasil!$K$6:$K$139,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"v3")</f>
         <v/>
       </c>
       <c r="F17" s="6">
@@ -1766,7 +1766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M139"/>
+  <dimension ref="A1:M144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10642,9 +10642,344 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="25" t="inlineStr">
+        <is>
+          <t>BR-135</t>
+        </is>
+      </c>
+      <c r="B140" s="26" t="inlineStr">
+        <is>
+          <t>Inflação</t>
+        </is>
+      </c>
+      <c r="C140" s="26" t="inlineStr">
+        <is>
+          <t>Aberturas</t>
+        </is>
+      </c>
+      <c r="D140" s="27" t="inlineStr">
+        <is>
+          <t>IPCA — Comercializáveis (tradables)</t>
+        </is>
+      </c>
+      <c r="E140" s="26" t="inlineStr">
+        <is>
+          <t>BCB SGS</t>
+        </is>
+      </c>
+      <c r="F140" s="26" t="inlineStr">
+        <is>
+          <t>4447</t>
+        </is>
+      </c>
+      <c r="G140" s="26" t="inlineStr">
+        <is>
+          <t>Mensal</t>
+        </is>
+      </c>
+      <c r="H140" s="26" t="inlineStr">
+        <is>
+          <t>% m/m</t>
+        </is>
+      </c>
+      <c r="I140" s="26" t="inlineStr">
+        <is>
+          <t>Var % mensal</t>
+        </is>
+      </c>
+      <c r="J140" s="26" t="inlineStr">
+        <is>
+          <t>Mensal, acum. 3/6/9/12m (encadeado), 3m/6m anualizado, YoY via 12m</t>
+        </is>
+      </c>
+      <c r="K140" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L140" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M140" s="26" t="inlineStr">
+        <is>
+          <t>Classificação do BCB; título oficial conferido no SGS em 2026-10-15. Preços formados no mercado internacional; reagem a câmbio e commodities</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="25" t="inlineStr">
+        <is>
+          <t>BR-136</t>
+        </is>
+      </c>
+      <c r="B141" s="26" t="inlineStr">
+        <is>
+          <t>Inflação</t>
+        </is>
+      </c>
+      <c r="C141" s="26" t="inlineStr">
+        <is>
+          <t>Aberturas</t>
+        </is>
+      </c>
+      <c r="D141" s="27" t="inlineStr">
+        <is>
+          <t>IPCA — Não comercializáveis</t>
+        </is>
+      </c>
+      <c r="E141" s="26" t="inlineStr">
+        <is>
+          <t>BCB SGS</t>
+        </is>
+      </c>
+      <c r="F141" s="26" t="inlineStr">
+        <is>
+          <t>4448</t>
+        </is>
+      </c>
+      <c r="G141" s="26" t="inlineStr">
+        <is>
+          <t>Mensal</t>
+        </is>
+      </c>
+      <c r="H141" s="26" t="inlineStr">
+        <is>
+          <t>% m/m</t>
+        </is>
+      </c>
+      <c r="I141" s="26" t="inlineStr">
+        <is>
+          <t>Var % mensal</t>
+        </is>
+      </c>
+      <c r="J141" s="26" t="inlineStr">
+        <is>
+          <t>Mensal, acum. 3/6/9/12m (encadeado), 3m/6m anualizado, YoY via 12m</t>
+        </is>
+      </c>
+      <c r="K141" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L141" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M141" s="26" t="inlineStr">
+        <is>
+          <t>Classificação do BCB; título oficial conferido no SGS em 2026-10-15. Preços formados no mercado doméstico; reagem a renda e demanda interna</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="25" t="inlineStr">
+        <is>
+          <t>BR-137</t>
+        </is>
+      </c>
+      <c r="B142" s="26" t="inlineStr">
+        <is>
+          <t>Inflação</t>
+        </is>
+      </c>
+      <c r="C142" s="26" t="inlineStr">
+        <is>
+          <t>Aberturas</t>
+        </is>
+      </c>
+      <c r="D142" s="27" t="inlineStr">
+        <is>
+          <t>IPCA — Bens duráveis</t>
+        </is>
+      </c>
+      <c r="E142" s="26" t="inlineStr">
+        <is>
+          <t>BCB SGS</t>
+        </is>
+      </c>
+      <c r="F142" s="26" t="inlineStr">
+        <is>
+          <t>10843</t>
+        </is>
+      </c>
+      <c r="G142" s="26" t="inlineStr">
+        <is>
+          <t>Mensal</t>
+        </is>
+      </c>
+      <c r="H142" s="26" t="inlineStr">
+        <is>
+          <t>% m/m</t>
+        </is>
+      </c>
+      <c r="I142" s="26" t="inlineStr">
+        <is>
+          <t>Var % mensal</t>
+        </is>
+      </c>
+      <c r="J142" s="26" t="inlineStr">
+        <is>
+          <t>Mensal, acum. 3/6/9/12m (encadeado), 3m/6m anualizado, YoY via 12m</t>
+        </is>
+      </c>
+      <c r="K142" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L142" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M142" s="26" t="inlineStr">
+        <is>
+          <t>Classificação do BCB; título oficial conferido no SGS em 2026-10-15. Compras em geral financiadas (veículos, eletrodomésticos); sensíveis a crédito, juros e câmbio</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="25" t="inlineStr">
+        <is>
+          <t>BR-138</t>
+        </is>
+      </c>
+      <c r="B143" s="26" t="inlineStr">
+        <is>
+          <t>Inflação</t>
+        </is>
+      </c>
+      <c r="C143" s="26" t="inlineStr">
+        <is>
+          <t>Aberturas</t>
+        </is>
+      </c>
+      <c r="D143" s="27" t="inlineStr">
+        <is>
+          <t>IPCA — Bens semiduráveis</t>
+        </is>
+      </c>
+      <c r="E143" s="26" t="inlineStr">
+        <is>
+          <t>BCB SGS</t>
+        </is>
+      </c>
+      <c r="F143" s="26" t="inlineStr">
+        <is>
+          <t>10842</t>
+        </is>
+      </c>
+      <c r="G143" s="26" t="inlineStr">
+        <is>
+          <t>Mensal</t>
+        </is>
+      </c>
+      <c r="H143" s="26" t="inlineStr">
+        <is>
+          <t>% m/m</t>
+        </is>
+      </c>
+      <c r="I143" s="26" t="inlineStr">
+        <is>
+          <t>Var % mensal</t>
+        </is>
+      </c>
+      <c r="J143" s="26" t="inlineStr">
+        <is>
+          <t>Mensal, acum. 3/6/9/12m (encadeado), 3m/6m anualizado, YoY via 12m</t>
+        </is>
+      </c>
+      <c r="K143" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L143" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M143" s="26" t="inlineStr">
+        <is>
+          <t>Classificação do BCB; título oficial conferido no SGS em 2026-10-15. Vestuário, calçados e similares</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="25" t="inlineStr">
+        <is>
+          <t>BR-139</t>
+        </is>
+      </c>
+      <c r="B144" s="26" t="inlineStr">
+        <is>
+          <t>Inflação</t>
+        </is>
+      </c>
+      <c r="C144" s="26" t="inlineStr">
+        <is>
+          <t>Aberturas</t>
+        </is>
+      </c>
+      <c r="D144" s="27" t="inlineStr">
+        <is>
+          <t>IPCA — Bens não duráveis</t>
+        </is>
+      </c>
+      <c r="E144" s="26" t="inlineStr">
+        <is>
+          <t>BCB SGS</t>
+        </is>
+      </c>
+      <c r="F144" s="26" t="inlineStr">
+        <is>
+          <t>10841</t>
+        </is>
+      </c>
+      <c r="G144" s="26" t="inlineStr">
+        <is>
+          <t>Mensal</t>
+        </is>
+      </c>
+      <c r="H144" s="26" t="inlineStr">
+        <is>
+          <t>% m/m</t>
+        </is>
+      </c>
+      <c r="I144" s="26" t="inlineStr">
+        <is>
+          <t>Var % mensal</t>
+        </is>
+      </c>
+      <c r="J144" s="26" t="inlineStr">
+        <is>
+          <t>Mensal, acum. 3/6/9/12m (encadeado), 3m/6m anualizado, YoY via 12m</t>
+        </is>
+      </c>
+      <c r="K144" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L144" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M144" s="26" t="inlineStr">
+        <is>
+          <t>Classificação do BCB; título oficial conferido no SGS em 2026-10-15. Alimentos, higiene, combustíveis e similares</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:M139"/>
-  <conditionalFormatting sqref="L6:L339">
+  <autoFilter ref="A5:M144"/>
+  <conditionalFormatting sqref="L6:L344">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L6="Verificado"</formula>
     </cfRule>
@@ -10667,16 +11002,16 @@
       <formula>$L6="Curado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K339">
+  <conditionalFormatting sqref="K6:K344">
     <cfRule type="expression" priority="8" dxfId="7">
       <formula>$K6="MVP"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K6:K339" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K344" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MVP,EUA,v2,v3"</formula1>
     </dataValidation>
-    <dataValidation sqref="L6:L339" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L6:L344" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Verificado,Confirmar,A mapear,Sem API,Pago,Derivado,Curado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Notícias oficiais por RSS (BCB, IBGE, Fed): adapter com fixtures reais e catálogo BR-140
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y547LUMzE2tZ8HqSCTt7kq
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Fontes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$145</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EUA'!$A$5:$M$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Central'!$A$5:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fontes'!$A$5:$F$25</definedName>
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -993,19 +993,19 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A7,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F7" s="6">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="I7" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$144,H7)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$145,H7)</f>
         <v/>
       </c>
     </row>
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A8,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F8" s="6">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="I8" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$144,H8)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$145,H8)</f>
         <v/>
       </c>
     </row>
@@ -1065,19 +1065,19 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A9,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F9" s="6">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="I9" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$144,H9)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$145,H9)</f>
         <v/>
       </c>
     </row>
@@ -1101,19 +1101,19 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A10,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F10" s="6">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="I10" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$144,H10)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$145,H10)</f>
         <v/>
       </c>
     </row>
@@ -1137,19 +1137,19 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A11,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F11" s="6">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="I11" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$144,H11)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$145,H11)</f>
         <v/>
       </c>
     </row>
@@ -1173,19 +1173,19 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A12,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F12" s="6">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="I12" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$144,H12)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$145,H12)</f>
         <v/>
       </c>
     </row>
@@ -1209,19 +1209,19 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A13,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F13" s="6">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="I13" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$144,H13)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$145,H13)</f>
         <v/>
       </c>
     </row>
@@ -1245,19 +1245,19 @@
         </is>
       </c>
       <c r="B14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A14,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F14" s="6">
@@ -1272,19 +1272,19 @@
         </is>
       </c>
       <c r="B15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A15,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F15" s="6">
@@ -1299,19 +1299,19 @@
         </is>
       </c>
       <c r="B16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A16,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F16" s="6">
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"MVP")</f>
         <v/>
       </c>
       <c r="C17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"EUA")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"v2")</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$144,$A17,Brasil!$K$6:$K$144,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"v3")</f>
         <v/>
       </c>
       <c r="F17" s="6">
@@ -1347,121 +1347,112 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="B18" s="16">
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"MVP")</f>
+        <v/>
+      </c>
+      <c r="C18" s="16">
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"EUA")</f>
+        <v/>
+      </c>
+      <c r="D18" s="16">
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"v2")</f>
+        <v/>
+      </c>
+      <c r="E18" s="16">
+        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"v3")</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>SUM(B18:E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B18" s="6">
-        <f>SUM(B7:B17)</f>
+      <c r="B19" s="6">
+        <f>SUM(B7:B18)</f>
         <v/>
       </c>
-      <c r="C18" s="6">
-        <f>SUM(C7:C17)</f>
+      <c r="C19" s="6">
+        <f>SUM(C7:C18)</f>
         <v/>
       </c>
-      <c r="D18" s="6">
-        <f>SUM(D7:D17)</f>
+      <c r="D19" s="6">
+        <f>SUM(D7:D18)</f>
         <v/>
       </c>
-      <c r="E18" s="6">
-        <f>SUM(E7:E17)</f>
+      <c r="E19" s="6">
+        <f>SUM(E7:E18)</f>
         <v/>
       </c>
-      <c r="F18" s="6">
-        <f>SUM(F7:F17)</f>
+      <c r="F19" s="6">
+        <f>SUM(F7:F18)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>EUA</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Aba</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>EUA</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>v2</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>v3</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="H22" s="15" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I21" s="15" t="inlineStr">
+      <c r="I22" s="15" t="inlineStr">
         <is>
           <t>Qtd</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>Mercado de Trabalho</t>
-        </is>
-      </c>
-      <c r="B22" s="16">
-        <f>COUNTIFS(EUA!$B$6:$B$101,$A22,EUA!$K$6:$K$101,"MVP")</f>
-        <v/>
-      </c>
-      <c r="C22" s="16">
-        <f>COUNTIFS(EUA!$B$6:$B$101,$A22,EUA!$K$6:$K$101,"EUA")</f>
-        <v/>
-      </c>
-      <c r="D22" s="16">
-        <f>COUNTIFS(EUA!$B$6:$B$101,$A22,EUA!$K$6:$K$101,"v2")</f>
-        <v/>
-      </c>
-      <c r="E22" s="16">
-        <f>COUNTIFS(EUA!$B$6:$B$101,$A22,EUA!$K$6:$K$101,"v3")</f>
-        <v/>
-      </c>
-      <c r="F22" s="6">
-        <f>SUM(B22:E22)</f>
-        <v/>
-      </c>
-      <c r="H22" s="17" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="I22" s="16">
-        <f>COUNTIF(EUA!$L$6:$L$101,H22)</f>
-        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Inflação</t>
+          <t>Mercado de Trabalho</t>
         </is>
       </c>
       <c r="B23" s="16">
@@ -1484,9 +1475,9 @@
         <f>SUM(B23:E23)</f>
         <v/>
       </c>
-      <c r="H23" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="I23" s="16">
@@ -1497,7 +1488,7 @@
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>Atividade</t>
+          <t>Inflação</t>
         </is>
       </c>
       <c r="B24" s="16">
@@ -1520,9 +1511,9 @@
         <f>SUM(B24:E24)</f>
         <v/>
       </c>
-      <c r="H24" s="19" t="inlineStr">
-        <is>
-          <t>A mapear</t>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
         </is>
       </c>
       <c r="I24" s="16">
@@ -1533,7 +1524,7 @@
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>Fed &amp; Juros</t>
+          <t>Atividade</t>
         </is>
       </c>
       <c r="B25" s="16">
@@ -1556,9 +1547,9 @@
         <f>SUM(B25:E25)</f>
         <v/>
       </c>
-      <c r="H25" s="20" t="inlineStr">
-        <is>
-          <t>Sem API</t>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>A mapear</t>
         </is>
       </c>
       <c r="I25" s="16">
@@ -1569,7 +1560,7 @@
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>Imobiliário</t>
+          <t>Fed &amp; Juros</t>
         </is>
       </c>
       <c r="B26" s="16">
@@ -1592,9 +1583,9 @@
         <f>SUM(B26:E26)</f>
         <v/>
       </c>
-      <c r="H26" s="21" t="inlineStr">
-        <is>
-          <t>Pago</t>
+      <c r="H26" s="20" t="inlineStr">
+        <is>
+          <t>Sem API</t>
         </is>
       </c>
       <c r="I26" s="16">
@@ -1605,7 +1596,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>Consumidor</t>
+          <t>Imobiliário</t>
         </is>
       </c>
       <c r="B27" s="16">
@@ -1628,9 +1619,9 @@
         <f>SUM(B27:E27)</f>
         <v/>
       </c>
-      <c r="H27" s="22" t="inlineStr">
-        <is>
-          <t>Derivado</t>
+      <c r="H27" s="21" t="inlineStr">
+        <is>
+          <t>Pago</t>
         </is>
       </c>
       <c r="I27" s="16">
@@ -1641,7 +1632,7 @@
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Corporativo</t>
+          <t>Consumidor</t>
         </is>
       </c>
       <c r="B28" s="16">
@@ -1664,9 +1655,9 @@
         <f>SUM(B28:E28)</f>
         <v/>
       </c>
-      <c r="H28" s="23" t="inlineStr">
-        <is>
-          <t>Curado</t>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>Derivado</t>
         </is>
       </c>
       <c r="I28" s="16">
@@ -1677,7 +1668,7 @@
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>Setor Externo &amp; Fiscal</t>
+          <t>Corporativo</t>
         </is>
       </c>
       <c r="B29" s="16">
@@ -1700,11 +1691,20 @@
         <f>SUM(B29:E29)</f>
         <v/>
       </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>Curado</t>
+        </is>
+      </c>
+      <c r="I29" s="16">
+        <f>COUNTIF(EUA!$L$6:$L$101,H29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>Risco &amp; Mercado</t>
+          <t>Setor Externo &amp; Fiscal</t>
         </is>
       </c>
       <c r="B30" s="16">
@@ -1729,29 +1729,56 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Risco &amp; Mercado</t>
+        </is>
+      </c>
+      <c r="B31" s="16">
+        <f>COUNTIFS(EUA!$B$6:$B$101,$A31,EUA!$K$6:$K$101,"MVP")</f>
+        <v/>
+      </c>
+      <c r="C31" s="16">
+        <f>COUNTIFS(EUA!$B$6:$B$101,$A31,EUA!$K$6:$K$101,"EUA")</f>
+        <v/>
+      </c>
+      <c r="D31" s="16">
+        <f>COUNTIFS(EUA!$B$6:$B$101,$A31,EUA!$K$6:$K$101,"v2")</f>
+        <v/>
+      </c>
+      <c r="E31" s="16">
+        <f>COUNTIFS(EUA!$B$6:$B$101,$A31,EUA!$K$6:$K$101,"v3")</f>
+        <v/>
+      </c>
+      <c r="F31" s="6">
+        <f>SUM(B31:E31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B31" s="6">
-        <f>SUM(B22:B30)</f>
+      <c r="B32" s="6">
+        <f>SUM(B23:B31)</f>
         <v/>
       </c>
-      <c r="C31" s="6">
-        <f>SUM(C22:C30)</f>
+      <c r="C32" s="6">
+        <f>SUM(C23:C31)</f>
         <v/>
       </c>
-      <c r="D31" s="6">
-        <f>SUM(D22:D30)</f>
+      <c r="D32" s="6">
+        <f>SUM(D23:D31)</f>
         <v/>
       </c>
-      <c r="E31" s="6">
-        <f>SUM(E22:E30)</f>
+      <c r="E32" s="6">
+        <f>SUM(E23:E31)</f>
         <v/>
       </c>
-      <c r="F31" s="6">
-        <f>SUM(F22:F30)</f>
+      <c r="F32" s="6">
+        <f>SUM(F23:F31)</f>
         <v/>
       </c>
     </row>
@@ -1766,7 +1793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M144"/>
+  <dimension ref="A1:M145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10977,9 +11004,76 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="25" t="inlineStr">
+        <is>
+          <t>BR-140</t>
+        </is>
+      </c>
+      <c r="B145" s="26" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C145" s="26" t="inlineStr">
+        <is>
+          <t>Notícias</t>
+        </is>
+      </c>
+      <c r="D145" s="27" t="inlineStr">
+        <is>
+          <t>Notícias oficiais: BCB (notas e notícias), IBGE e Fed</t>
+        </is>
+      </c>
+      <c r="E145" s="26" t="inlineStr">
+        <is>
+          <t>RSS oficial</t>
+        </is>
+      </c>
+      <c r="F145" s="26" t="inlineStr">
+        <is>
+          <t>bcb_notas ; bcb_noticias ; ibge ; fed</t>
+        </is>
+      </c>
+      <c r="G145" s="26" t="inlineStr">
+        <is>
+          <t>Contínua</t>
+        </is>
+      </c>
+      <c r="H145" s="26" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="I145" s="26" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="J145" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K145" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L145" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M145" s="26" t="inlineStr">
+        <is>
+          <t>Feeds RSS/Atom oficiais (BCB sitefeeds, Agência IBGE, Federal Reserve press_monetary); título e resumo em texto puro na tabela events (tipo noticia); fixtures reais gravadas em 2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:M144"/>
-  <conditionalFormatting sqref="L6:L344">
+  <autoFilter ref="A5:M145"/>
+  <conditionalFormatting sqref="L6:L345">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L6="Verificado"</formula>
     </cfRule>
@@ -11002,16 +11096,16 @@
       <formula>$L6="Curado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K344">
+  <conditionalFormatting sqref="K6:K345">
     <cfRule type="expression" priority="8" dxfId="7">
       <formula>$K6="MVP"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K6:K344" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K345" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MVP,EUA,v2,v3"</formula1>
     </dataValidation>
-    <dataValidation sqref="L6:L344" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L6:L345" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Verificado,Confirmar,A mapear,Sem API,Pago,Derivado,Curado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Agenda de divulgações do IBGE pela API oficial de calendário (BR-141)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y547LUMzE2tZ8HqSCTt7kq
</commit_message>
<xml_diff>
--- a/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
+++ b/docs/catalogo/Argus_Catalogo_de_Dados.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Fontes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brasil'!$A$5:$M$146</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EUA'!$A$5:$M$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Central'!$A$5:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fontes'!$A$5:$F$25</definedName>
@@ -993,19 +993,19 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A7,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A7,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A7,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A7,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A7,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F7" s="6">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="I7" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$145,H7)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$146,H7)</f>
         <v/>
       </c>
     </row>
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A8,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A8,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A8,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A8,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A8,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F8" s="6">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="I8" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$145,H8)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$146,H8)</f>
         <v/>
       </c>
     </row>
@@ -1065,19 +1065,19 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A9,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A9,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A9,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A9,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A9,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F9" s="6">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="I9" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$145,H9)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$146,H9)</f>
         <v/>
       </c>
     </row>
@@ -1101,19 +1101,19 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A10,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A10,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A10,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A10,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A10,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F10" s="6">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="I10" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$145,H10)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$146,H10)</f>
         <v/>
       </c>
     </row>
@@ -1137,19 +1137,19 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A11,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A11,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A11,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A11,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A11,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F11" s="6">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="I11" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$145,H11)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$146,H11)</f>
         <v/>
       </c>
     </row>
@@ -1173,19 +1173,19 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A12,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A12,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A12,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A12,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A12,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F12" s="6">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="I12" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$145,H12)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$146,H12)</f>
         <v/>
       </c>
     </row>
@@ -1209,19 +1209,19 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A13,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A13,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A13,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E13" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A13,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A13,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F13" s="6">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="I13" s="16">
-        <f>COUNTIF(Brasil!$L$6:$L$145,H13)</f>
+        <f>COUNTIF(Brasil!$L$6:$L$146,H13)</f>
         <v/>
       </c>
     </row>
@@ -1245,19 +1245,19 @@
         </is>
       </c>
       <c r="B14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A14,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A14,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A14,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E14" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A14,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A14,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F14" s="6">
@@ -1272,19 +1272,19 @@
         </is>
       </c>
       <c r="B15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A15,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A15,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A15,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E15" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A15,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A15,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F15" s="6">
@@ -1299,19 +1299,19 @@
         </is>
       </c>
       <c r="B16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A16,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A16,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A16,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A16,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A16,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F16" s="6">
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A17,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A17,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A17,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A17,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A17,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F17" s="6">
@@ -1353,19 +1353,19 @@
         </is>
       </c>
       <c r="B18" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"MVP")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A18,Brasil!$K$6:$K$146,"MVP")</f>
         <v/>
       </c>
       <c r="C18" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"EUA")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A18,Brasil!$K$6:$K$146,"EUA")</f>
         <v/>
       </c>
       <c r="D18" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"v2")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A18,Brasil!$K$6:$K$146,"v2")</f>
         <v/>
       </c>
       <c r="E18" s="16">
-        <f>COUNTIFS(Brasil!$B$6:$B$145,$A18,Brasil!$K$6:$K$145,"v3")</f>
+        <f>COUNTIFS(Brasil!$B$6:$B$146,$A18,Brasil!$K$6:$K$146,"v3")</f>
         <v/>
       </c>
       <c r="F18" s="6">
@@ -1793,7 +1793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M145"/>
+  <dimension ref="A1:M146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11071,9 +11071,76 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="25" t="inlineStr">
+        <is>
+          <t>BR-141</t>
+        </is>
+      </c>
+      <c r="B146" s="26" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C146" s="26" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="D146" s="27" t="inlineStr">
+        <is>
+          <t>Agenda de divulgações do IBGE (IPCA, IPCA-15, PNAD, PIM, PMC, PMS, PIB, LSPA)</t>
+        </is>
+      </c>
+      <c r="E146" s="26" t="inlineStr">
+        <is>
+          <t>IBGE calendário (servicodados v3)</t>
+        </is>
+      </c>
+      <c r="F146" s="26" t="inlineStr">
+        <is>
+          <t>calendario</t>
+        </is>
+      </c>
+      <c r="G146" s="26" t="inlineStr">
+        <is>
+          <t>Contínua</t>
+        </is>
+      </c>
+      <c r="H146" s="26" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="I146" s="26" t="inlineStr">
+        <is>
+          <t>Evento</t>
+        </is>
+      </c>
+      <c r="J146" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K146" s="26" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L146" s="26" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="M146" s="26" t="inlineStr">
+        <is>
+          <t>API oficial de calendário do IBGE (servicodados/api/v3/calendario), janela de 120 dias; resposta real gravada em 2026-10-19; vai para a tabela events (tipo agenda)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:M145"/>
-  <conditionalFormatting sqref="L6:L345">
+  <autoFilter ref="A5:M146"/>
+  <conditionalFormatting sqref="L6:L346">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L6="Verificado"</formula>
     </cfRule>
@@ -11096,16 +11163,16 @@
       <formula>$L6="Curado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K345">
+  <conditionalFormatting sqref="K6:K346">
     <cfRule type="expression" priority="8" dxfId="7">
       <formula>$K6="MVP"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K6:K345" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K346" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MVP,EUA,v2,v3"</formula1>
     </dataValidation>
-    <dataValidation sqref="L6:L345" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L6:L346" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Verificado,Confirmar,A mapear,Sem API,Pago,Derivado,Curado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>